<commit_message>
release: prepare Sector 0.93 candidate
</commit_message>
<xml_diff>
--- a/docs/sector_v093_decision_register.xlsx
+++ b/docs/sector_v093_decision_register.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A17EAA8-14B0-4671-97FF-2384AD0EAFAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{94A9AD7A-E071-45EA-8DAC-26AD93BD4E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" xr2:uid="{72B71BF4-87E9-4839-9757-643C29FE9B68}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C2A185B3-B91E-4EDE-B8CE-CE8CAEEA21C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="5" r:id="rId1"/>
@@ -562,52 +562,52 @@
     <t>v0.92 baseline</t>
   </si>
   <si>
+    <t>Merged</t>
+  </si>
+  <si>
+    <t>PR-02 - Bridge scope reset, schema 24 and design-standard registry</t>
+  </si>
+  <si>
+    <t>PR-01</t>
+  </si>
+  <si>
+    <t>PR-03 - Textbook worked calculations and complete substitutions</t>
+  </si>
+  <si>
+    <t>PR-04 - Input correctness, reusable IDs and mathematical table guides</t>
+  </si>
+  <si>
+    <t>PR-05 - Stateful input tabs and explicit modelled direction</t>
+  </si>
+  <si>
+    <t>PR-06 - Optional crack criterion and DK/NA heightened check</t>
+  </si>
+  <si>
+    <t>PR-03, PR-04, PR-05</t>
+  </si>
+  <si>
+    <t>PR-07A - Eurocode-style shared equation renderer</t>
+  </si>
+  <si>
+    <t>PR-03</t>
+  </si>
+  <si>
+    <t>PR-07B - Manual/report information architecture and profiles</t>
+  </si>
+  <si>
+    <t>PR-06, PR-07A</t>
+  </si>
+  <si>
+    <t>PR-08 - Double-click portable Windows packaging</t>
+  </si>
+  <si>
+    <t>PR-09 - Full qualification and Sector 0.93 release</t>
+  </si>
+  <si>
+    <t>PR-01 through PR-08</t>
+  </si>
+  <si>
     <t>In progress</t>
-  </si>
-  <si>
-    <t>PR-02 - Bridge scope reset, schema 24 and design-standard registry</t>
-  </si>
-  <si>
-    <t>PR-01</t>
-  </si>
-  <si>
-    <t>Planned</t>
-  </si>
-  <si>
-    <t>PR-03 - Textbook calculation evidence and complete substitutions</t>
-  </si>
-  <si>
-    <t>PR-04 - Input correctness, reusable IDs and mathematical table guides</t>
-  </si>
-  <si>
-    <t>PR-05 - Stateful input tabs and explicit modelled direction</t>
-  </si>
-  <si>
-    <t>PR-06 - Optional crack criterion and DK/NA heightened check</t>
-  </si>
-  <si>
-    <t>PR-03, PR-04, PR-05</t>
-  </si>
-  <si>
-    <t>PR-07A - Eurocode-style shared equation renderer</t>
-  </si>
-  <si>
-    <t>PR-03</t>
-  </si>
-  <si>
-    <t>PR-07B - Manual/report information architecture and profiles</t>
-  </si>
-  <si>
-    <t>PR-06, PR-07A</t>
-  </si>
-  <si>
-    <t>PR-08 - Double-click portable Windows packaging</t>
-  </si>
-  <si>
-    <t>PR-09 - Full qualification and Sector 0.93 release</t>
-  </si>
-  <si>
-    <t>PR-01 through PR-08</t>
   </si>
   <si>
     <t>Standards status and implementation boundary</t>
@@ -881,7 +881,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -921,12 +921,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2F0D9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -973,7 +967,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1012,9 +1006,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1617,66 +1608,66 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1215A3BF-D210-4957-A975-727D65CA3B0B}" name="RegisterMetadata" displayName="RegisterMetadata" ref="A4:B12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="27">
-  <autoFilter ref="A4:B12" xr:uid="{1215A3BF-D210-4957-A975-727D65CA3B0B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D75A2600-4D04-41EC-9D52-75B39D5D7B0B}" name="RegisterMetadata" displayName="RegisterMetadata" ref="A4:B12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="27">
+  <autoFilter ref="A4:B12" xr:uid="{D75A2600-4D04-41EC-9D52-75B39D5D7B0B}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{92C78141-E3B1-4AB9-912D-BFD739507178}" name="Record" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{A8635C14-11DA-4105-8950-6328807C7104}" name="Value" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{52F455FE-0371-436A-BF2E-D42278D30322}" name="Record" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{E5F50F42-3C77-49D6-AE91-AB549B625A63}" name="Value" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{814CBAB8-883C-4E22-BF18-C3E3D9CD6839}" name="V093Decisions" displayName="V093Decisions" ref="A4:G31" totalsRowShown="0" headerRowDxfId="26" dataDxfId="23">
-  <autoFilter ref="A4:G31" xr:uid="{814CBAB8-883C-4E22-BF18-C3E3D9CD6839}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E0C9D7ED-BEAC-4899-BA11-59FBF9EB3E11}" name="V093Decisions" displayName="V093Decisions" ref="A4:G31" totalsRowShown="0" headerRowDxfId="26" dataDxfId="23">
+  <autoFilter ref="A4:G31" xr:uid="{E0C9D7ED-BEAC-4899-BA11-59FBF9EB3E11}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0333F55B-8EA6-4BE2-9342-73A9B366A75A}" name="Decision ID" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{D6F71AE0-327A-43AE-9601-FE248B0A7551}" name="Frozen decision" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{FA3E9B36-B142-440C-B9F6-E7E99A18E110}" name="Reason and boundary" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{4FE4C691-1C5D-4F09-8973-81DD21B0C301}" name="Acceptance evidence" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{B368773B-E800-4F67-8DD2-D2C35ACF0301}" name="Owning PR" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{31FE8135-471B-4647-8748-70A662086C4F}" name="Status" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{A5D1A95F-47F0-405F-80B0-38F127F19574}" name="Disposition" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{18D6C0A3-67D2-4269-98CE-CBBCD6F261BD}" name="Decision ID" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{BA807BE6-9CA0-4C2E-9025-893654A719EC}" name="Frozen decision" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{A9CDA27A-86C6-4A0A-8D40-88C9DAB05760}" name="Reason and boundary" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{3E6A9323-136A-45EC-9A6B-8C33AE84A211}" name="Acceptance evidence" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{65B3FA64-605C-4C06-899E-08478FAF429B}" name="Owning PR" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{53731860-2803-406E-9B65-8D76C93903AF}" name="Status" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{6674E16E-CAD1-4EF4-AD87-6A272BD7182A}" name="Disposition" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CEDC65F0-9EC1-4AED-B9BB-28378C75FDAE}" name="V093Programme" displayName="V093Programme" ref="A4:D14" totalsRowShown="0" headerRowDxfId="17" dataDxfId="14">
-  <autoFilter ref="A4:D14" xr:uid="{CEDC65F0-9EC1-4AED-B9BB-28378C75FDAE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D7FEB7AE-E1B4-41D1-9158-81A7B34222C7}" name="V093Programme" displayName="V093Programme" ref="A4:D14" totalsRowShown="0" headerRowDxfId="17" dataDxfId="14">
+  <autoFilter ref="A4:D14" xr:uid="{D7FEB7AE-E1B4-41D1-9158-81A7B34222C7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C85248DE-7F2B-4FA3-84D2-3A39BA95F24A}" name="Order" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{EBD9AB9F-D458-449D-8D99-D57C64BECFBA}" name="Slice" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{B033388B-3B1E-4EC4-A1F5-FA4C1A9FBF6F}" name="Depends on" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{F0EF9893-E97C-4728-99FE-31E5CC8B498B}" name="Status" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{00BDFE26-5C4A-47B3-830C-5E326ECD09DC}" name="Order" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{5A932A5F-50DA-4B3F-AD95-D7C3C74A1FF8}" name="Slice" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{3B28D4D3-C9C5-4506-BA12-AC8E42961B60}" name="Depends on" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{7231A709-3C5E-4C31-AF6B-ED04E1411BC3}" name="Status" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{151F08DE-437C-4DF5-B6B4-E439CE47B208}" name="V093Standards" displayName="V093Standards" ref="A4:D8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="6">
-  <autoFilter ref="A4:D8" xr:uid="{151F08DE-437C-4DF5-B6B4-E439CE47B208}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A22342A4-6C71-43AC-827D-27FB08F967BD}" name="V093Standards" displayName="V093Standards" ref="A4:D8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="6">
+  <autoFilter ref="A4:D8" xr:uid="{A22342A4-6C71-43AC-827D-27FB08F967BD}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{A872C289-6F37-4C9F-B0CD-30C43BEE80B6}" name="Family" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{9DCBCBB7-4E97-449C-88A4-17EC2132DA1B}" name="Sector label and scope" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{3218F1A5-6231-49A0-88E6-34EF08ABD79B}" name="Status disclosure" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{F07D2C17-C471-4B64-AF49-A114F968C6BA}" name="v0.93 boundary" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{1DB29296-9BDD-4546-AEDC-D772A2DA9AAE}" name="Family" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{FC1DD4AB-962D-429D-950B-590FE5FDECA8}" name="Sector label and scope" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{9B5F966F-4D6D-4F79-871A-F7AE78F6C3E9}" name="Status disclosure" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{A3677AE0-65F6-49B2-8220-AF1145811EC5}" name="v0.93 boundary" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E3C3CD4D-3DA8-46D7-ABC7-55A971D48D22}" name="V093PublicationQA" displayName="V093PublicationQA" ref="A4:D19" totalsRowShown="0" headerRowDxfId="5" dataDxfId="2">
-  <autoFilter ref="A4:D19" xr:uid="{E3C3CD4D-3DA8-46D7-ABC7-55A971D48D22}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6DFD6F99-54C2-423F-8B5A-40F5D0F97C52}" name="V093PublicationQA" displayName="V093PublicationQA" ref="A4:D19" totalsRowShown="0" headerRowDxfId="5" dataDxfId="2">
+  <autoFilter ref="A4:D19" xr:uid="{6DFD6F99-54C2-423F-8B5A-40F5D0F97C52}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{3D7B0CD9-6BEE-4A14-BA9D-A85358E8AF04}" name="Surface" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{45C8089D-B4A1-424F-BA27-CA187BDB5A75}" name="Current page" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{4C6ABB85-3CA6-4E99-9B12-107B96D7ED42}" name="Observed issue" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{2DC27603-8F2F-4C8F-B135-5351B51C351F}" name="Required treatment" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{BD9DFB0F-A694-49B6-A0FC-D6DBDFBA9437}" name="Surface" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{F25BDDBC-5E0D-4144-85CB-D06CC1AB55C9}" name="Current page" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{9B476978-2D85-4A33-83B2-27478ED875E9}" name="Observed issue" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{8492889E-1EE0-4208-95A6-C5751A98895A}" name="Required treatment" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1998,7 +1989,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07EEBA17-7425-452D-B753-084C766FA1FE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDDC0FF0-BD95-4B8E-9BE1-B0B110D66704}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2106,7 +2097,7 @@
       </c>
       <c r="E8" s="8">
         <f>COUNTIF('PR Programme'!D5:D14,"Planned")</f>
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2205,7 +2196,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B21E74F-5A7A-402F-BA78-CB6D9C29921D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C366E68D-BB7D-41B6-B190-E4C8C327CBFC}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2908,7 +2899,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26F07102-CA2B-4EB0-8A5C-032FD2FFAB66}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6F11020-E627-4531-B156-1B8198BA06A4}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2961,7 +2952,7 @@
       <c r="C5" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="12" t="s">
         <v>170</v>
       </c>
     </row>
@@ -2975,8 +2966,8 @@
       <c r="C6" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>173</v>
+      <c r="D6" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2984,13 +2975,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="D7" s="14" t="s">
-        <v>173</v>
+      <c r="D7" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2998,13 +2989,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="14" t="s">
-        <v>173</v>
+      <c r="D8" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3012,13 +3003,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="14" t="s">
-        <v>173</v>
+      <c r="D9" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3026,13 +3017,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>173</v>
+      <c r="D10" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3040,13 +3031,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>173</v>
+      <c r="D11" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3054,13 +3045,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>173</v>
+      <c r="D12" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3068,13 +3059,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="14" t="s">
-        <v>173</v>
+      <c r="D13" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3082,13 +3073,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="13" t="s">
         <v>185</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -3109,7 +3100,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13083F5F-131B-444D-9F50-205CCE18186B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC1A1289-E16F-4DE3-93B2-9E175235B449}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3226,7 +3217,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E011D655-07DE-44E2-AB83-0C81FE84EC11}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F27FAC5-996E-4F32-B7C3-5BAF77861788}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>

<commit_message>
PR-09: qualify Sector 0.93 release candidate (#391)
Close the approved v0.93 PR programme as an authenticated release candidate while preserving schema 24, unsigned portable boundaries, exact QA evidence, and draft-only publication semantics.
</commit_message>
<xml_diff>
--- a/docs/sector_v093_decision_register.xlsx
+++ b/docs/sector_v093_decision_register.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A17EAA8-14B0-4671-97FF-2384AD0EAFAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{94A9AD7A-E071-45EA-8DAC-26AD93BD4E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" xr2:uid="{72B71BF4-87E9-4839-9757-643C29FE9B68}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C2A185B3-B91E-4EDE-B8CE-CE8CAEEA21C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="5" r:id="rId1"/>
@@ -562,52 +562,52 @@
     <t>v0.92 baseline</t>
   </si>
   <si>
+    <t>Merged</t>
+  </si>
+  <si>
+    <t>PR-02 - Bridge scope reset, schema 24 and design-standard registry</t>
+  </si>
+  <si>
+    <t>PR-01</t>
+  </si>
+  <si>
+    <t>PR-03 - Textbook worked calculations and complete substitutions</t>
+  </si>
+  <si>
+    <t>PR-04 - Input correctness, reusable IDs and mathematical table guides</t>
+  </si>
+  <si>
+    <t>PR-05 - Stateful input tabs and explicit modelled direction</t>
+  </si>
+  <si>
+    <t>PR-06 - Optional crack criterion and DK/NA heightened check</t>
+  </si>
+  <si>
+    <t>PR-03, PR-04, PR-05</t>
+  </si>
+  <si>
+    <t>PR-07A - Eurocode-style shared equation renderer</t>
+  </si>
+  <si>
+    <t>PR-03</t>
+  </si>
+  <si>
+    <t>PR-07B - Manual/report information architecture and profiles</t>
+  </si>
+  <si>
+    <t>PR-06, PR-07A</t>
+  </si>
+  <si>
+    <t>PR-08 - Double-click portable Windows packaging</t>
+  </si>
+  <si>
+    <t>PR-09 - Full qualification and Sector 0.93 release</t>
+  </si>
+  <si>
+    <t>PR-01 through PR-08</t>
+  </si>
+  <si>
     <t>In progress</t>
-  </si>
-  <si>
-    <t>PR-02 - Bridge scope reset, schema 24 and design-standard registry</t>
-  </si>
-  <si>
-    <t>PR-01</t>
-  </si>
-  <si>
-    <t>Planned</t>
-  </si>
-  <si>
-    <t>PR-03 - Textbook calculation evidence and complete substitutions</t>
-  </si>
-  <si>
-    <t>PR-04 - Input correctness, reusable IDs and mathematical table guides</t>
-  </si>
-  <si>
-    <t>PR-05 - Stateful input tabs and explicit modelled direction</t>
-  </si>
-  <si>
-    <t>PR-06 - Optional crack criterion and DK/NA heightened check</t>
-  </si>
-  <si>
-    <t>PR-03, PR-04, PR-05</t>
-  </si>
-  <si>
-    <t>PR-07A - Eurocode-style shared equation renderer</t>
-  </si>
-  <si>
-    <t>PR-03</t>
-  </si>
-  <si>
-    <t>PR-07B - Manual/report information architecture and profiles</t>
-  </si>
-  <si>
-    <t>PR-06, PR-07A</t>
-  </si>
-  <si>
-    <t>PR-08 - Double-click portable Windows packaging</t>
-  </si>
-  <si>
-    <t>PR-09 - Full qualification and Sector 0.93 release</t>
-  </si>
-  <si>
-    <t>PR-01 through PR-08</t>
   </si>
   <si>
     <t>Standards status and implementation boundary</t>
@@ -881,7 +881,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -921,12 +921,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2F0D9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -973,7 +967,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1012,9 +1006,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1617,66 +1608,66 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1215A3BF-D210-4957-A975-727D65CA3B0B}" name="RegisterMetadata" displayName="RegisterMetadata" ref="A4:B12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="27">
-  <autoFilter ref="A4:B12" xr:uid="{1215A3BF-D210-4957-A975-727D65CA3B0B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D75A2600-4D04-41EC-9D52-75B39D5D7B0B}" name="RegisterMetadata" displayName="RegisterMetadata" ref="A4:B12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="27">
+  <autoFilter ref="A4:B12" xr:uid="{D75A2600-4D04-41EC-9D52-75B39D5D7B0B}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{92C78141-E3B1-4AB9-912D-BFD739507178}" name="Record" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{A8635C14-11DA-4105-8950-6328807C7104}" name="Value" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{52F455FE-0371-436A-BF2E-D42278D30322}" name="Record" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{E5F50F42-3C77-49D6-AE91-AB549B625A63}" name="Value" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{814CBAB8-883C-4E22-BF18-C3E3D9CD6839}" name="V093Decisions" displayName="V093Decisions" ref="A4:G31" totalsRowShown="0" headerRowDxfId="26" dataDxfId="23">
-  <autoFilter ref="A4:G31" xr:uid="{814CBAB8-883C-4E22-BF18-C3E3D9CD6839}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E0C9D7ED-BEAC-4899-BA11-59FBF9EB3E11}" name="V093Decisions" displayName="V093Decisions" ref="A4:G31" totalsRowShown="0" headerRowDxfId="26" dataDxfId="23">
+  <autoFilter ref="A4:G31" xr:uid="{E0C9D7ED-BEAC-4899-BA11-59FBF9EB3E11}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0333F55B-8EA6-4BE2-9342-73A9B366A75A}" name="Decision ID" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{D6F71AE0-327A-43AE-9601-FE248B0A7551}" name="Frozen decision" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{FA3E9B36-B142-440C-B9F6-E7E99A18E110}" name="Reason and boundary" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{4FE4C691-1C5D-4F09-8973-81DD21B0C301}" name="Acceptance evidence" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{B368773B-E800-4F67-8DD2-D2C35ACF0301}" name="Owning PR" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{31FE8135-471B-4647-8748-70A662086C4F}" name="Status" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{A5D1A95F-47F0-405F-80B0-38F127F19574}" name="Disposition" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{18D6C0A3-67D2-4269-98CE-CBBCD6F261BD}" name="Decision ID" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{BA807BE6-9CA0-4C2E-9025-893654A719EC}" name="Frozen decision" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{A9CDA27A-86C6-4A0A-8D40-88C9DAB05760}" name="Reason and boundary" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{3E6A9323-136A-45EC-9A6B-8C33AE84A211}" name="Acceptance evidence" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{65B3FA64-605C-4C06-899E-08478FAF429B}" name="Owning PR" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{53731860-2803-406E-9B65-8D76C93903AF}" name="Status" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{6674E16E-CAD1-4EF4-AD87-6A272BD7182A}" name="Disposition" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CEDC65F0-9EC1-4AED-B9BB-28378C75FDAE}" name="V093Programme" displayName="V093Programme" ref="A4:D14" totalsRowShown="0" headerRowDxfId="17" dataDxfId="14">
-  <autoFilter ref="A4:D14" xr:uid="{CEDC65F0-9EC1-4AED-B9BB-28378C75FDAE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D7FEB7AE-E1B4-41D1-9158-81A7B34222C7}" name="V093Programme" displayName="V093Programme" ref="A4:D14" totalsRowShown="0" headerRowDxfId="17" dataDxfId="14">
+  <autoFilter ref="A4:D14" xr:uid="{D7FEB7AE-E1B4-41D1-9158-81A7B34222C7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C85248DE-7F2B-4FA3-84D2-3A39BA95F24A}" name="Order" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{EBD9AB9F-D458-449D-8D99-D57C64BECFBA}" name="Slice" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{B033388B-3B1E-4EC4-A1F5-FA4C1A9FBF6F}" name="Depends on" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{F0EF9893-E97C-4728-99FE-31E5CC8B498B}" name="Status" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{00BDFE26-5C4A-47B3-830C-5E326ECD09DC}" name="Order" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{5A932A5F-50DA-4B3F-AD95-D7C3C74A1FF8}" name="Slice" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{3B28D4D3-C9C5-4506-BA12-AC8E42961B60}" name="Depends on" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{7231A709-3C5E-4C31-AF6B-ED04E1411BC3}" name="Status" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{151F08DE-437C-4DF5-B6B4-E439CE47B208}" name="V093Standards" displayName="V093Standards" ref="A4:D8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="6">
-  <autoFilter ref="A4:D8" xr:uid="{151F08DE-437C-4DF5-B6B4-E439CE47B208}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A22342A4-6C71-43AC-827D-27FB08F967BD}" name="V093Standards" displayName="V093Standards" ref="A4:D8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="6">
+  <autoFilter ref="A4:D8" xr:uid="{A22342A4-6C71-43AC-827D-27FB08F967BD}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{A872C289-6F37-4C9F-B0CD-30C43BEE80B6}" name="Family" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{9DCBCBB7-4E97-449C-88A4-17EC2132DA1B}" name="Sector label and scope" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{3218F1A5-6231-49A0-88E6-34EF08ABD79B}" name="Status disclosure" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{F07D2C17-C471-4B64-AF49-A114F968C6BA}" name="v0.93 boundary" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{1DB29296-9BDD-4546-AEDC-D772A2DA9AAE}" name="Family" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{FC1DD4AB-962D-429D-950B-590FE5FDECA8}" name="Sector label and scope" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{9B5F966F-4D6D-4F79-871A-F7AE78F6C3E9}" name="Status disclosure" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{A3677AE0-65F6-49B2-8220-AF1145811EC5}" name="v0.93 boundary" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E3C3CD4D-3DA8-46D7-ABC7-55A971D48D22}" name="V093PublicationQA" displayName="V093PublicationQA" ref="A4:D19" totalsRowShown="0" headerRowDxfId="5" dataDxfId="2">
-  <autoFilter ref="A4:D19" xr:uid="{E3C3CD4D-3DA8-46D7-ABC7-55A971D48D22}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6DFD6F99-54C2-423F-8B5A-40F5D0F97C52}" name="V093PublicationQA" displayName="V093PublicationQA" ref="A4:D19" totalsRowShown="0" headerRowDxfId="5" dataDxfId="2">
+  <autoFilter ref="A4:D19" xr:uid="{6DFD6F99-54C2-423F-8B5A-40F5D0F97C52}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{3D7B0CD9-6BEE-4A14-BA9D-A85358E8AF04}" name="Surface" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{45C8089D-B4A1-424F-BA27-CA187BDB5A75}" name="Current page" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{4C6ABB85-3CA6-4E99-9B12-107B96D7ED42}" name="Observed issue" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{2DC27603-8F2F-4C8F-B135-5351B51C351F}" name="Required treatment" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{BD9DFB0F-A694-49B6-A0FC-D6DBDFBA9437}" name="Surface" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{F25BDDBC-5E0D-4144-85CB-D06CC1AB55C9}" name="Current page" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{9B476978-2D85-4A33-83B2-27478ED875E9}" name="Observed issue" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{8492889E-1EE0-4208-95A6-C5751A98895A}" name="Required treatment" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1998,7 +1989,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07EEBA17-7425-452D-B753-084C766FA1FE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDDC0FF0-BD95-4B8E-9BE1-B0B110D66704}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2106,7 +2097,7 @@
       </c>
       <c r="E8" s="8">
         <f>COUNTIF('PR Programme'!D5:D14,"Planned")</f>
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2205,7 +2196,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B21E74F-5A7A-402F-BA78-CB6D9C29921D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C366E68D-BB7D-41B6-B190-E4C8C327CBFC}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2908,7 +2899,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26F07102-CA2B-4EB0-8A5C-032FD2FFAB66}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6F11020-E627-4531-B156-1B8198BA06A4}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2961,7 +2952,7 @@
       <c r="C5" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="12" t="s">
         <v>170</v>
       </c>
     </row>
@@ -2975,8 +2966,8 @@
       <c r="C6" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>173</v>
+      <c r="D6" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2984,13 +2975,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="D7" s="14" t="s">
-        <v>173</v>
+      <c r="D7" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2998,13 +2989,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="14" t="s">
-        <v>173</v>
+      <c r="D8" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3012,13 +3003,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="14" t="s">
-        <v>173</v>
+      <c r="D9" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3026,13 +3017,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>173</v>
+      <c r="D10" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3040,13 +3031,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>173</v>
+      <c r="D11" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3054,13 +3045,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>173</v>
+      <c r="D12" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3068,13 +3059,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="14" t="s">
-        <v>173</v>
+      <c r="D13" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3082,13 +3073,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="13" t="s">
         <v>185</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -3109,7 +3100,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13083F5F-131B-444D-9F50-205CCE18186B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC1A1289-E16F-4DE3-93B2-9E175235B449}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3226,7 +3217,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E011D655-07DE-44E2-AB83-0C81FE84EC11}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F27FAC5-996E-4F32-B7C3-5BAF77861788}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>

<commit_message>
docs: close Sector 0.93 release programme
</commit_message>
<xml_diff>
--- a/docs/sector_v093_decision_register.xlsx
+++ b/docs/sector_v093_decision_register.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94A9AD7A-E071-45EA-8DAC-26AD93BD4E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C5A6F5D-77B5-48A7-8555-BB0B2DB8E814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C2A185B3-B91E-4EDE-B8CE-CE8CAEEA21C3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{63BC7C18-72B2-4966-BEC9-0B8D68CF5471}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="5" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="251">
   <si>
     <t>Sector v0.93 Decision Register</t>
   </si>
@@ -605,9 +605,6 @@
   </si>
   <si>
     <t>PR-01 through PR-08</t>
-  </si>
-  <si>
-    <t>In progress</t>
   </si>
   <si>
     <t>Standards status and implementation boundary</t>
@@ -1608,66 +1605,66 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D75A2600-4D04-41EC-9D52-75B39D5D7B0B}" name="RegisterMetadata" displayName="RegisterMetadata" ref="A4:B12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="27">
-  <autoFilter ref="A4:B12" xr:uid="{D75A2600-4D04-41EC-9D52-75B39D5D7B0B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{769C12E5-B7E8-494E-9A65-2075D2306A99}" name="RegisterMetadata" displayName="RegisterMetadata" ref="A4:B12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="27">
+  <autoFilter ref="A4:B12" xr:uid="{769C12E5-B7E8-494E-9A65-2075D2306A99}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{52F455FE-0371-436A-BF2E-D42278D30322}" name="Record" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{E5F50F42-3C77-49D6-AE91-AB549B625A63}" name="Value" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{CB04BFC9-590B-412D-891A-28212CCECFAC}" name="Record" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{3A124376-BFD6-4AD0-B4B3-86EB9B7A249B}" name="Value" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E0C9D7ED-BEAC-4899-BA11-59FBF9EB3E11}" name="V093Decisions" displayName="V093Decisions" ref="A4:G31" totalsRowShown="0" headerRowDxfId="26" dataDxfId="23">
-  <autoFilter ref="A4:G31" xr:uid="{E0C9D7ED-BEAC-4899-BA11-59FBF9EB3E11}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{402E0365-B590-4F7E-9991-BBD617DEF910}" name="V093Decisions" displayName="V093Decisions" ref="A4:G31" totalsRowShown="0" headerRowDxfId="26" dataDxfId="23">
+  <autoFilter ref="A4:G31" xr:uid="{402E0365-B590-4F7E-9991-BBD617DEF910}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{18D6C0A3-67D2-4269-98CE-CBBCD6F261BD}" name="Decision ID" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{BA807BE6-9CA0-4C2E-9025-893654A719EC}" name="Frozen decision" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{A9CDA27A-86C6-4A0A-8D40-88C9DAB05760}" name="Reason and boundary" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{3E6A9323-136A-45EC-9A6B-8C33AE84A211}" name="Acceptance evidence" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{65B3FA64-605C-4C06-899E-08478FAF429B}" name="Owning PR" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{53731860-2803-406E-9B65-8D76C93903AF}" name="Status" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{6674E16E-CAD1-4EF4-AD87-6A272BD7182A}" name="Disposition" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{D59960F1-7608-46FF-B737-79F5D776CA9F}" name="Decision ID" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{87BBD414-0EEF-4375-B8FC-BF97647B665F}" name="Frozen decision" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{CD7CE841-5F85-44E8-8A3F-3F369712DFAB}" name="Reason and boundary" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{81581489-7399-49A7-83A3-F6E774D7845C}" name="Acceptance evidence" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{EBDD7CE3-8037-43F2-ABB3-56E5A2DEDF85}" name="Owning PR" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{2E01A201-5471-4C0F-AA45-C03D4B3FCD9D}" name="Status" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{715F2481-7E51-4D11-8AEE-6CC4F9A73390}" name="Disposition" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D7FEB7AE-E1B4-41D1-9158-81A7B34222C7}" name="V093Programme" displayName="V093Programme" ref="A4:D14" totalsRowShown="0" headerRowDxfId="17" dataDxfId="14">
-  <autoFilter ref="A4:D14" xr:uid="{D7FEB7AE-E1B4-41D1-9158-81A7B34222C7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B6273181-F218-433C-B8DD-86C11FE1B51E}" name="V093Programme" displayName="V093Programme" ref="A4:D14" totalsRowShown="0" headerRowDxfId="17" dataDxfId="14">
+  <autoFilter ref="A4:D14" xr:uid="{B6273181-F218-433C-B8DD-86C11FE1B51E}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00BDFE26-5C4A-47B3-830C-5E326ECD09DC}" name="Order" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{5A932A5F-50DA-4B3F-AD95-D7C3C74A1FF8}" name="Slice" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{3B28D4D3-C9C5-4506-BA12-AC8E42961B60}" name="Depends on" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{7231A709-3C5E-4C31-AF6B-ED04E1411BC3}" name="Status" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{1ED5DCDE-C57F-4121-9C0C-E4A7A9F013E6}" name="Order" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{FB618EDD-CD21-4F0B-8964-DFE6859A1245}" name="Slice" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{E4586875-FB6E-4A98-90C5-92EAD805D0CE}" name="Depends on" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{F25D5CFA-F66D-4FEC-8E7E-D71374D94891}" name="Status" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A22342A4-6C71-43AC-827D-27FB08F967BD}" name="V093Standards" displayName="V093Standards" ref="A4:D8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="6">
-  <autoFilter ref="A4:D8" xr:uid="{A22342A4-6C71-43AC-827D-27FB08F967BD}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D77E9B64-D2AD-4F5A-A6C5-AA67A987E4EB}" name="V093Standards" displayName="V093Standards" ref="A4:D8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="6">
+  <autoFilter ref="A4:D8" xr:uid="{D77E9B64-D2AD-4F5A-A6C5-AA67A987E4EB}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{1DB29296-9BDD-4546-AEDC-D772A2DA9AAE}" name="Family" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{FC1DD4AB-962D-429D-950B-590FE5FDECA8}" name="Sector label and scope" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{9B5F966F-4D6D-4F79-871A-F7AE78F6C3E9}" name="Status disclosure" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{A3677AE0-65F6-49B2-8220-AF1145811EC5}" name="v0.93 boundary" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{DD590290-945F-47EF-A8CC-FC72FAFE0FC4}" name="Family" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{7AB975C2-2BD2-4A0F-B11E-253971AA1F4A}" name="Sector label and scope" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{CF9D2B9D-7309-49D1-BA53-5D731FE610D2}" name="Status disclosure" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{1FE9A358-D0C3-401A-A15D-04883B871D53}" name="v0.93 boundary" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6DFD6F99-54C2-423F-8B5A-40F5D0F97C52}" name="V093PublicationQA" displayName="V093PublicationQA" ref="A4:D19" totalsRowShown="0" headerRowDxfId="5" dataDxfId="2">
-  <autoFilter ref="A4:D19" xr:uid="{6DFD6F99-54C2-423F-8B5A-40F5D0F97C52}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{BA704E92-AFD5-4C62-80C4-0F99FAB3AD58}" name="V093PublicationQA" displayName="V093PublicationQA" ref="A4:D19" totalsRowShown="0" headerRowDxfId="5" dataDxfId="2">
+  <autoFilter ref="A4:D19" xr:uid="{BA704E92-AFD5-4C62-80C4-0F99FAB3AD58}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{BD9DFB0F-A694-49B6-A0FC-D6DBDFBA9437}" name="Surface" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{F25BDDBC-5E0D-4144-85CB-D06CC1AB55C9}" name="Current page" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{9B476978-2D85-4A33-83B2-27478ED875E9}" name="Observed issue" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{8492889E-1EE0-4208-95A6-C5751A98895A}" name="Required treatment" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{65CFBB5D-50B6-4CBD-A7A1-9495878DD0A6}" name="Surface" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{C9B50A61-EE53-46D3-9691-8640E129DF65}" name="Current page" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{14481BEE-FBDC-48E9-8FF2-AC6FD00BB891}" name="Observed issue" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{8C00059B-57A7-43C7-ADA2-135F5A15AA4C}" name="Required treatment" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1989,7 +1986,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDDC0FF0-BD95-4B8E-9BE1-B0B110D66704}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B13546DE-DEBD-4D8F-AB4E-04166B74DE08}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2112,7 +2109,7 @@
       </c>
       <c r="E9" s="8">
         <f>COUNTIF('PR Programme'!D5:D14,"In progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2196,7 +2193,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C366E68D-BB7D-41B6-B190-E4C8C327CBFC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{169EBB2E-AB1F-41AA-B21A-EFD55A060FB1}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2899,7 +2896,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6F11020-E627-4531-B156-1B8198BA06A4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{986EBBF6-C8BD-415D-8C47-5F19C18C863D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3078,8 +3075,8 @@
       <c r="C14" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>185</v>
+      <c r="D14" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -3100,7 +3097,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC1A1289-E16F-4DE3-93B2-9E175235B449}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32BC4F4F-B574-43EF-9AE2-41678665BE60}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3115,7 +3112,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3123,7 +3120,7 @@
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3131,72 +3128,72 @@
     </row>
     <row r="4" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>194</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>202</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>206</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -3217,7 +3214,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F27FAC5-996E-4F32-B7C3-5BAF77861788}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9D838BA-E56D-4787-93DF-CEA46CB6DD99}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3232,7 +3229,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3240,7 +3237,7 @@
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3248,226 +3245,226 @@
     </row>
     <row r="4" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>212</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B5" s="4">
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>215</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B6" s="4">
         <v>2</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>217</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B7" s="4">
         <v>11</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>222</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>225</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B10" s="4">
         <v>41</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>227</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>230</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B12" s="4">
         <v>2</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>233</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>236</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>239</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B15" s="4">
         <v>42</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>241</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B16" s="4">
         <v>43</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>243</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="4" t="s">
         <v>246</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B18" s="4">
         <v>55</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>248</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B19" s="4">
         <v>56</v>
       </c>
       <c r="C19" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>250</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PR-09: close Sector 0.93 release-readiness programme (#396)
</commit_message>
<xml_diff>
--- a/docs/sector_v093_decision_register.xlsx
+++ b/docs/sector_v093_decision_register.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94A9AD7A-E071-45EA-8DAC-26AD93BD4E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C5A6F5D-77B5-48A7-8555-BB0B2DB8E814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C2A185B3-B91E-4EDE-B8CE-CE8CAEEA21C3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{63BC7C18-72B2-4966-BEC9-0B8D68CF5471}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="5" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="251">
   <si>
     <t>Sector v0.93 Decision Register</t>
   </si>
@@ -605,9 +605,6 @@
   </si>
   <si>
     <t>PR-01 through PR-08</t>
-  </si>
-  <si>
-    <t>In progress</t>
   </si>
   <si>
     <t>Standards status and implementation boundary</t>
@@ -1608,66 +1605,66 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D75A2600-4D04-41EC-9D52-75B39D5D7B0B}" name="RegisterMetadata" displayName="RegisterMetadata" ref="A4:B12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="27">
-  <autoFilter ref="A4:B12" xr:uid="{D75A2600-4D04-41EC-9D52-75B39D5D7B0B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{769C12E5-B7E8-494E-9A65-2075D2306A99}" name="RegisterMetadata" displayName="RegisterMetadata" ref="A4:B12" totalsRowShown="0" headerRowDxfId="30" dataDxfId="27">
+  <autoFilter ref="A4:B12" xr:uid="{769C12E5-B7E8-494E-9A65-2075D2306A99}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{52F455FE-0371-436A-BF2E-D42278D30322}" name="Record" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{E5F50F42-3C77-49D6-AE91-AB549B625A63}" name="Value" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{CB04BFC9-590B-412D-891A-28212CCECFAC}" name="Record" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{3A124376-BFD6-4AD0-B4B3-86EB9B7A249B}" name="Value" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E0C9D7ED-BEAC-4899-BA11-59FBF9EB3E11}" name="V093Decisions" displayName="V093Decisions" ref="A4:G31" totalsRowShown="0" headerRowDxfId="26" dataDxfId="23">
-  <autoFilter ref="A4:G31" xr:uid="{E0C9D7ED-BEAC-4899-BA11-59FBF9EB3E11}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{402E0365-B590-4F7E-9991-BBD617DEF910}" name="V093Decisions" displayName="V093Decisions" ref="A4:G31" totalsRowShown="0" headerRowDxfId="26" dataDxfId="23">
+  <autoFilter ref="A4:G31" xr:uid="{402E0365-B590-4F7E-9991-BBD617DEF910}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{18D6C0A3-67D2-4269-98CE-CBBCD6F261BD}" name="Decision ID" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{BA807BE6-9CA0-4C2E-9025-893654A719EC}" name="Frozen decision" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{A9CDA27A-86C6-4A0A-8D40-88C9DAB05760}" name="Reason and boundary" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{3E6A9323-136A-45EC-9A6B-8C33AE84A211}" name="Acceptance evidence" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{65B3FA64-605C-4C06-899E-08478FAF429B}" name="Owning PR" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{53731860-2803-406E-9B65-8D76C93903AF}" name="Status" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{6674E16E-CAD1-4EF4-AD87-6A272BD7182A}" name="Disposition" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{D59960F1-7608-46FF-B737-79F5D776CA9F}" name="Decision ID" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{87BBD414-0EEF-4375-B8FC-BF97647B665F}" name="Frozen decision" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{CD7CE841-5F85-44E8-8A3F-3F369712DFAB}" name="Reason and boundary" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{81581489-7399-49A7-83A3-F6E774D7845C}" name="Acceptance evidence" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{EBDD7CE3-8037-43F2-ABB3-56E5A2DEDF85}" name="Owning PR" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{2E01A201-5471-4C0F-AA45-C03D4B3FCD9D}" name="Status" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{715F2481-7E51-4D11-8AEE-6CC4F9A73390}" name="Disposition" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D7FEB7AE-E1B4-41D1-9158-81A7B34222C7}" name="V093Programme" displayName="V093Programme" ref="A4:D14" totalsRowShown="0" headerRowDxfId="17" dataDxfId="14">
-  <autoFilter ref="A4:D14" xr:uid="{D7FEB7AE-E1B4-41D1-9158-81A7B34222C7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B6273181-F218-433C-B8DD-86C11FE1B51E}" name="V093Programme" displayName="V093Programme" ref="A4:D14" totalsRowShown="0" headerRowDxfId="17" dataDxfId="14">
+  <autoFilter ref="A4:D14" xr:uid="{B6273181-F218-433C-B8DD-86C11FE1B51E}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00BDFE26-5C4A-47B3-830C-5E326ECD09DC}" name="Order" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{5A932A5F-50DA-4B3F-AD95-D7C3C74A1FF8}" name="Slice" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{3B28D4D3-C9C5-4506-BA12-AC8E42961B60}" name="Depends on" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{7231A709-3C5E-4C31-AF6B-ED04E1411BC3}" name="Status" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{1ED5DCDE-C57F-4121-9C0C-E4A7A9F013E6}" name="Order" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{FB618EDD-CD21-4F0B-8964-DFE6859A1245}" name="Slice" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{E4586875-FB6E-4A98-90C5-92EAD805D0CE}" name="Depends on" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{F25D5CFA-F66D-4FEC-8E7E-D71374D94891}" name="Status" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A22342A4-6C71-43AC-827D-27FB08F967BD}" name="V093Standards" displayName="V093Standards" ref="A4:D8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="6">
-  <autoFilter ref="A4:D8" xr:uid="{A22342A4-6C71-43AC-827D-27FB08F967BD}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D77E9B64-D2AD-4F5A-A6C5-AA67A987E4EB}" name="V093Standards" displayName="V093Standards" ref="A4:D8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="6">
+  <autoFilter ref="A4:D8" xr:uid="{D77E9B64-D2AD-4F5A-A6C5-AA67A987E4EB}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{1DB29296-9BDD-4546-AEDC-D772A2DA9AAE}" name="Family" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{FC1DD4AB-962D-429D-950B-590FE5FDECA8}" name="Sector label and scope" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{9B5F966F-4D6D-4F79-871A-F7AE78F6C3E9}" name="Status disclosure" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{A3677AE0-65F6-49B2-8220-AF1145811EC5}" name="v0.93 boundary" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{DD590290-945F-47EF-A8CC-FC72FAFE0FC4}" name="Family" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{7AB975C2-2BD2-4A0F-B11E-253971AA1F4A}" name="Sector label and scope" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{CF9D2B9D-7309-49D1-BA53-5D731FE610D2}" name="Status disclosure" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{1FE9A358-D0C3-401A-A15D-04883B871D53}" name="v0.93 boundary" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6DFD6F99-54C2-423F-8B5A-40F5D0F97C52}" name="V093PublicationQA" displayName="V093PublicationQA" ref="A4:D19" totalsRowShown="0" headerRowDxfId="5" dataDxfId="2">
-  <autoFilter ref="A4:D19" xr:uid="{6DFD6F99-54C2-423F-8B5A-40F5D0F97C52}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{BA704E92-AFD5-4C62-80C4-0F99FAB3AD58}" name="V093PublicationQA" displayName="V093PublicationQA" ref="A4:D19" totalsRowShown="0" headerRowDxfId="5" dataDxfId="2">
+  <autoFilter ref="A4:D19" xr:uid="{BA704E92-AFD5-4C62-80C4-0F99FAB3AD58}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{BD9DFB0F-A694-49B6-A0FC-D6DBDFBA9437}" name="Surface" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{F25BDDBC-5E0D-4144-85CB-D06CC1AB55C9}" name="Current page" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{9B476978-2D85-4A33-83B2-27478ED875E9}" name="Observed issue" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{8492889E-1EE0-4208-95A6-C5751A98895A}" name="Required treatment" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{65CFBB5D-50B6-4CBD-A7A1-9495878DD0A6}" name="Surface" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{C9B50A61-EE53-46D3-9691-8640E129DF65}" name="Current page" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{14481BEE-FBDC-48E9-8FF2-AC6FD00BB891}" name="Observed issue" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{8C00059B-57A7-43C7-ADA2-135F5A15AA4C}" name="Required treatment" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1989,7 +1986,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDDC0FF0-BD95-4B8E-9BE1-B0B110D66704}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B13546DE-DEBD-4D8F-AB4E-04166B74DE08}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2112,7 +2109,7 @@
       </c>
       <c r="E9" s="8">
         <f>COUNTIF('PR Programme'!D5:D14,"In progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2196,7 +2193,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C366E68D-BB7D-41B6-B190-E4C8C327CBFC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{169EBB2E-AB1F-41AA-B21A-EFD55A060FB1}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2899,7 +2896,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6F11020-E627-4531-B156-1B8198BA06A4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{986EBBF6-C8BD-415D-8C47-5F19C18C863D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3078,8 +3075,8 @@
       <c r="C14" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>185</v>
+      <c r="D14" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -3100,7 +3097,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC1A1289-E16F-4DE3-93B2-9E175235B449}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32BC4F4F-B574-43EF-9AE2-41678665BE60}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3115,7 +3112,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3123,7 +3120,7 @@
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3131,72 +3128,72 @@
     </row>
     <row r="4" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>194</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>202</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>206</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -3217,7 +3214,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F27FAC5-996E-4F32-B7C3-5BAF77861788}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9D838BA-E56D-4787-93DF-CEA46CB6DD99}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3232,7 +3229,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3240,7 +3237,7 @@
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3248,226 +3245,226 @@
     </row>
     <row r="4" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>212</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B5" s="4">
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>215</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B6" s="4">
         <v>2</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>217</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B7" s="4">
         <v>11</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>222</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>225</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B10" s="4">
         <v>41</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>227</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>230</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B12" s="4">
         <v>2</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>233</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>236</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>239</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B15" s="4">
         <v>42</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>241</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B16" s="4">
         <v>43</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>243</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="4" t="s">
         <v>246</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B18" s="4">
         <v>55</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>248</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B19" s="4">
         <v>56</v>
       </c>
       <c r="C19" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>250</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>